<commit_message>
Daily attendance processing - 2026-03-20 16:52:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -622,7 +622,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023</t>
+          <t>2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023</t>
+          <t>2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-03-22 11:34:55 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -622,7 +622,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023</t>
+          <t>2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2022/2023, 2023/2024, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023</t>
+          <t>2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2022/2023, 2023/2024, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-11 13:59:06 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-13 12:15:17 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-14 21:22:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-15 09:59:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-15 14:12:15 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023, 2023/2024</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023, 2023/2024</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-16 00:11:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1741,7 +1741,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-16 08:12:38 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-16 16:09:32 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2023/2024, 2022/2023</t>
+          <t>2022/2023, 2025/2026, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-16 17:09:48 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-16 21:24:59 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-17 20:27:14 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2022/2023, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-18 10:09:27 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2025/2026, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2025/2026, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-20 17:50:51 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2022/2023, 2023/2024</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-21 07:05:57 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-22 18:30:28 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2025/2026, 2023/2024</t>
+          <t>2025/2026, 2023/2024, 2022/2023</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-23 11:05:17 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2022/2023, 2023/2024, 2025/2026</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-05-23 23:43:14 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
+++ b/attendance_reports/Y3_B2526_CNS_session_analysis.xlsx
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>2023/2024, 2025/2026, 2022/2023</t>
+          <t>2023/2024, 2022/2023, 2025/2026</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">

</xml_diff>